<commit_message>
feat(pipeline_lab): implement LLM prompt deduplication cache and test coverage
</commit_message>
<xml_diff>
--- a/pipeline_lab/output/populated_MEDIUM_datacenter_power_cooling_questions.xlsx
+++ b/pipeline_lab/output/populated_MEDIUM_datacenter_power_cooling_questions.xlsx
@@ -487,12 +487,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2 utility power feeds provide N+1 redundancy</t>
+          <t>Two utility power feeds provide N+1 redundancy at the facility level, each rated for 2.5 MW.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 3.2</t>
+          <t>Page 1, 1. Power Distribution</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 2.1</t>
+          <t>Page 1, Section 2. UPS Configuration</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2N topology per server hall</t>
+          <t>Each server hall has two fully independent UPS paths, either of which can carry the full hall load alone.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Text</t>
+          <t>Page 1, 2. UPS Configuration</t>
         </is>
       </c>
     </row>
@@ -538,12 +538,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Battery runtime at full load is 12 minutes.</t>
+          <t>Battery runtime at full load is 12 minutes, sufficient to bridge the approximately 45-second generator startup and transfer window with significant margin.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 2.2</t>
+          <t>Page 1, Section 2. UPS Configuration</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 3.2</t>
+          <t>Page 1, Section 3. Cooling Systems</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 4.1</t>
+          <t>Page 1, 4. Power Usage Effectiveness (PUE)</t>
         </is>
       </c>
     </row>
@@ -589,12 +589,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>The facility's target PUE is 1.25, and the current average PUE is 1.35, which is 0.1 higher than the target.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Page 1, Section 4.1</t>
+          <t>Page 1, Section 4. Power Usage Effectiveness (PUE)</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Hall D (new) has the least available IT load capacity remaining.</t>
+          <t>Hall B has the least available capacity remaining (190 kW).</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Hall D has 65 racks and uses In-row chilled water + rear-door heat exchangers for cooling.</t>
+          <t>Hall D has 65 racks, and it uses In-row chilled water + rear-door heat exchangers for cooling.</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Semi-annual service for all three chillers falls in the third week of next month</t>
+          <t>Chiller maintenance is semi-annual, with the next scheduled service for all three chillers falling in the third week of next month.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Page 2, Table T01-01</t>
+          <t>Page 2, Section 2. Maintenance Schedule</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Page 2, Section 4.1</t>
+          <t>NOT_SPECIFIED</t>
         </is>
       </c>
     </row>

</xml_diff>